<commit_message>
[REL69] Overprint and constraints (#801)
</commit_message>
<xml_diff>
--- a/docs/CHILI-GraFx/applications/editor-comparison/features.xlsx
+++ b/docs/CHILI-GraFx/applications/editor-comparison/features.xlsx
@@ -916,7 +916,7 @@
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C22" s="1" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="D22" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio: fill and stroke on text, shape and barcode frames in print intent — see [Overprint](/GraFx-Studio/concepts/overprint/)</t>
         </is>
       </c>
     </row>
@@ -3060,7 +3060,7 @@
       </c>
       <c r="D119" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio: image, text, shape and component frames — see [Constraints](/GraFx-Studio/concepts/constraints/)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[REL-74] Rich Text Format (#822)
</commit_message>
<xml_diff>
--- a/docs/CHILI-GraFx/applications/editor-comparison/features.xlsx
+++ b/docs/CHILI-GraFx/applications/editor-comparison/features.xlsx
@@ -3226,7 +3226,7 @@
       </c>
       <c r="B127" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>✅</t>
         </is>
       </c>
       <c r="C127" s="1" t="inlineStr">
@@ -3236,7 +3236,7 @@
       </c>
       <c r="D127" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>GraFx Studio: as a Rich text variable, with tags mapped to styles by rich text import rules — see [Rich text variables](/GraFx-Studio/guides/template-variables/rich-text/)</t>
         </is>
       </c>
     </row>
@@ -4644,7 +4644,7 @@
       </c>
       <c r="D191" s="1" t="inlineStr">
         <is>
-          <t>Not supported in templates that include components</t>
+          <t>GraFx Studio: Experimental, including component frames — see [Output to HTML](/GraFx-Studio/guides/output/html/)</t>
         </is>
       </c>
     </row>

</xml_diff>